<commit_message>
feat:Task 2 — Exploratory Data Analysis performed
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_unified_data_enriched.xlsx
+++ b/data/processed/ethiopia_fi_unified_data_enriched.xlsx
@@ -5241,10 +5241,8 @@
           <t>agents</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>2022-09-30</t>
-        </is>
+      <c r="L45" s="1" t="n">
+        <v>44834</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -5292,7 +5290,7 @@
       <c r="AD45" t="inlineStr"/>
       <c r="AE45" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
@@ -5357,10 +5355,8 @@
           <t>agents</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>2023-07-01</t>
-        </is>
+      <c r="L46" s="1" t="n">
+        <v>45108</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -5408,7 +5404,7 @@
       <c r="AD46" t="inlineStr"/>
       <c r="AE46" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF46" t="inlineStr">
@@ -5473,10 +5469,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>2023-06-30</t>
-        </is>
+      <c r="L47" s="1" t="n">
+        <v>45107</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -5524,7 +5518,7 @@
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
@@ -5589,10 +5583,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>2023-06-30</t>
-        </is>
+      <c r="L48" s="1" t="n">
+        <v>45107</v>
       </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
@@ -5640,7 +5632,7 @@
       <c r="AD48" t="inlineStr"/>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -5705,10 +5697,8 @@
           <t>loans</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>2023-07-01</t>
-        </is>
+      <c r="L49" s="1" t="n">
+        <v>45108</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
@@ -5756,7 +5746,7 @@
       <c r="AD49" t="inlineStr"/>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
@@ -5821,10 +5811,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>2023-01-15</t>
-        </is>
+      <c r="L50" s="1" t="n">
+        <v>44941</v>
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
@@ -5872,7 +5860,7 @@
       <c r="AD50" t="inlineStr"/>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -5937,10 +5925,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>2024-01-15</t>
-        </is>
+      <c r="L51" s="1" t="n">
+        <v>45306</v>
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
@@ -5988,7 +5974,7 @@
       <c r="AD51" t="inlineStr"/>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
@@ -6053,10 +6039,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
+      <c r="L52" s="1" t="n">
+        <v>46215</v>
       </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
@@ -6104,7 +6088,7 @@
       <c r="AD52" t="inlineStr"/>
       <c r="AE52" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF52" t="inlineStr">
@@ -6151,10 +6135,8 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>2023-10-09</t>
-        </is>
+      <c r="L53" s="1" t="n">
+        <v>45208</v>
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
@@ -6194,7 +6176,7 @@
       <c r="AD53" t="inlineStr"/>
       <c r="AE53" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF53" t="inlineStr">
@@ -6241,10 +6223,8 @@
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
+      <c r="L54" s="1" t="n">
+        <v>45804</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
@@ -6284,7 +6264,7 @@
       <c r="AD54" t="inlineStr"/>
       <c r="AE54" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF54" t="inlineStr">
@@ -6331,10 +6311,8 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>2023-09-01</t>
-        </is>
+      <c r="L55" s="1" t="n">
+        <v>45170</v>
       </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
@@ -6374,7 +6352,7 @@
       <c r="AD55" t="inlineStr"/>
       <c r="AE55" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF55" t="inlineStr">
@@ -6421,10 +6399,8 @@
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
+      <c r="L56" s="1" t="n">
+        <v>46215</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
@@ -6464,7 +6440,7 @@
       <c r="AD56" t="inlineStr"/>
       <c r="AE56" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AF56" t="inlineStr">
@@ -8390,7 +8366,7 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
@@ -8495,7 +8471,7 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
@@ -8596,7 +8572,7 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
@@ -8697,7 +8673,7 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
@@ -8798,7 +8774,7 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
@@ -8903,7 +8879,7 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Trainee</t>
+          <t>Yengusie Demilie Alene</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">

</xml_diff>

<commit_message>
updates: updates to task 5 for dashboard screenshots for README
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_unified_data_enriched.xlsx
+++ b/data/processed/ethiopia_fi_unified_data_enriched.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ethiopia_fi_unified_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ethiopia_fi_unified_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Impact_sheet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>